<commit_message>
KEY_Video_2: SV of "I [PUT] BUY PIZZA BASKET" is I BUY (USV); the later I BUY PIZZA is a Repeated SV
</commit_message>
<xml_diff>
--- a/reference_keys/KEY_Video_2.xlsx
+++ b/reference_keys/KEY_Video_2.xlsx
@@ -948,7 +948,7 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>USV:  I PUT</t>
+          <t>USV:  I BUY</t>
         </is>
       </c>
     </row>
@@ -1451,14 +1451,9 @@
           <t>Lexical Verb</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Unique Subject-Verb Combination (USV)</t>
-        </is>
-      </c>
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>USV:  I BUY</t>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Repeated SV Combination</t>
         </is>
       </c>
     </row>

</xml_diff>